<commit_message>
feat: Introduce new training program documentation for 'Assembleur Montage Câblage' and 'Chaudronnier d'atelier', and update the main index.
</commit_message>
<xml_diff>
--- a/OI/chaudronnier_datelier_prf_tpfp_ormocn_cei_tmi_bourges/Tableau de bord Kanban.xlsx
+++ b/OI/chaudronnier_datelier_prf_tpfp_ormocn_cei_tmi_bourges/Tableau de bord Kanban.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/chaudronnier_datelier_prf_tpfp_ormocn_cei_tmi_bourges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="8_{F7918DB6-62EF-48DD-BA2B-CE213045F091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{29D8540F-8C52-4A91-80B0-1A2C0038FC53}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{F7918DB6-62EF-48DD-BA2B-CE213045F091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5E1EDC5-8661-4024-8A0F-C3528DA7A373}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Graphique" sheetId="36" r:id="rId1"/>
@@ -503,6 +503,9 @@
                 <c:pt idx="1">
                   <c:v>1316</c:v>
                 </c:pt>
+                <c:pt idx="2">
+                  <c:v>1588</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -569,6 +572,9 @@
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1360</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1416</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2884,7 +2890,9 @@
       <c r="C14" s="17">
         <v>1316</v>
       </c>
-      <c r="D14" s="17"/>
+      <c r="D14" s="17">
+        <v>1588</v>
+      </c>
       <c r="E14" s="17"/>
     </row>
     <row r="15" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2897,7 +2905,9 @@
       <c r="C15" s="19">
         <v>1360</v>
       </c>
-      <c r="D15" s="19"/>
+      <c r="D15" s="19">
+        <v>1416</v>
+      </c>
       <c r="E15" s="19"/>
     </row>
     <row r="16" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
feat: Add Monteur Cableur training intervention email and Issoudun resources, updating index.html.
</commit_message>
<xml_diff>
--- a/OI/chaudronnier_datelier_prf_tpfp_ormocn_cei_tmi_bourges/Tableau de bord Kanban.xlsx
+++ b/OI/chaudronnier_datelier_prf_tpfp_ormocn_cei_tmi_bourges/Tableau de bord Kanban.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/chaudronnier_datelier_prf_tpfp_ormocn_cei_tmi_bourges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{F7918DB6-62EF-48DD-BA2B-CE213045F091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5E1EDC5-8661-4024-8A0F-C3528DA7A373}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="8_{F7918DB6-62EF-48DD-BA2B-CE213045F091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21A7E750-798F-416C-B139-58CFF5B40C97}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Graphique" sheetId="36" r:id="rId1"/>
@@ -299,7 +299,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -373,6 +373,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -391,7 +395,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -906,6 +910,9 @@
                 <c:pt idx="1">
                   <c:v>0.93500000000000005</c:v>
                 </c:pt>
+                <c:pt idx="2" formatCode="0%">
+                  <c:v>0.92</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -972,6 +979,9 @@
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.13</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.38</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1303,6 +1313,9 @@
                 <c:pt idx="1">
                   <c:v>0.67600000000000005</c:v>
                 </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.84199999999999997</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1369,6 +1382,9 @@
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.75</c:v>
+                </c:pt>
+                <c:pt idx="2" formatCode="0.0%">
+                  <c:v>0.82399999999999995</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2119,6 +2135,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
@@ -2500,21 +2520,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="26" t="s">
+      <c r="B1" s="25"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="27"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="23" t="s">
+      <c r="E1" s="28"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="24"/>
-      <c r="I1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="26"/>
     </row>
     <row r="2" spans="1:9" ht="5.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
@@ -2767,10 +2787,12 @@
       <c r="B3" s="10">
         <v>1</v>
       </c>
-      <c r="C3" s="29">
+      <c r="C3" s="23">
         <v>0.93500000000000005</v>
       </c>
-      <c r="D3" s="10"/>
+      <c r="D3" s="10">
+        <v>0.92</v>
+      </c>
       <c r="E3" s="10"/>
     </row>
     <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2783,7 +2805,9 @@
       <c r="C4" s="12">
         <v>0.13</v>
       </c>
-      <c r="D4" s="12"/>
+      <c r="D4" s="12">
+        <v>0.38</v>
+      </c>
       <c r="E4" s="12"/>
     </row>
     <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2820,10 +2844,12 @@
       <c r="B8" s="10">
         <v>0.71</v>
       </c>
-      <c r="C8" s="29">
+      <c r="C8" s="23">
         <v>0.67600000000000005</v>
       </c>
-      <c r="D8" s="10"/>
+      <c r="D8" s="23">
+        <v>0.84199999999999997</v>
+      </c>
       <c r="E8" s="10"/>
     </row>
     <row r="9" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2836,7 +2862,9 @@
       <c r="C9" s="12">
         <v>0.75</v>
       </c>
-      <c r="D9" s="12"/>
+      <c r="D9" s="30">
+        <v>0.82399999999999995</v>
+      </c>
       <c r="E9" s="12"/>
     </row>
     <row r="10" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
feat: Create initial resource page for Industrial Organization training in Issoudun.
</commit_message>
<xml_diff>
--- a/OI/chaudronnier_datelier_prf_tpfp_ormocn_cei_tmi_bourges/Tableau de bord Kanban.xlsx
+++ b/OI/chaudronnier_datelier_prf_tpfp_ormocn_cei_tmi_bourges/Tableau de bord Kanban.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/chaudronnier_datelier_prf_tpfp_ormocn_cei_tmi_bourges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="8_{F7918DB6-62EF-48DD-BA2B-CE213045F091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21A7E750-798F-416C-B139-58CFF5B40C97}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{F7918DB6-62EF-48DD-BA2B-CE213045F091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6748A3B0-1982-47C9-80FF-1115F6F65D3E}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Graphique" sheetId="36" r:id="rId1"/>
@@ -579,6 +579,9 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1416</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1548</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2936,7 +2939,9 @@
       <c r="D15" s="19">
         <v>1416</v>
       </c>
-      <c r="E15" s="19"/>
+      <c r="E15" s="19">
+        <v>1548</v>
+      </c>
     </row>
     <row r="16" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="13" t="s">

</xml_diff>

<commit_message>
feat: Implement NextAuth.js authentication with Discord and GitHub providers and tRPC integration.
</commit_message>
<xml_diff>
--- a/OI/chaudronnier_datelier_prf_tpfp_ormocn_cei_tmi_bourges/Tableau de bord Kanban.xlsx
+++ b/OI/chaudronnier_datelier_prf_tpfp_ormocn_cei_tmi_bourges/Tableau de bord Kanban.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/chaudronnier_datelier_prf_tpfp_ormocn_cei_tmi_bourges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{F7918DB6-62EF-48DD-BA2B-CE213045F091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6748A3B0-1982-47C9-80FF-1115F6F65D3E}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{F7918DB6-62EF-48DD-BA2B-CE213045F091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3401AE44-50ED-4F56-B4B9-EE802157FB83}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Graphique" sheetId="36" r:id="rId1"/>
@@ -509,6 +509,9 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1588</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1317</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2924,7 +2927,9 @@
       <c r="D14" s="17">
         <v>1588</v>
       </c>
-      <c r="E14" s="17"/>
+      <c r="E14" s="17">
+        <v>1317</v>
+      </c>
     </row>
     <row r="15" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="11" t="s">

</xml_diff>

<commit_message>
feat: add Kanban dashboard spreadsheet
</commit_message>
<xml_diff>
--- a/OI/chaudronnier_datelier_prf_tpfp_ormocn_cei_tmi_bourges/Tableau de bord Kanban.xlsx
+++ b/OI/chaudronnier_datelier_prf_tpfp_ormocn_cei_tmi_bourges/Tableau de bord Kanban.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/chaudronnier_datelier_prf_tpfp_ormocn_cei_tmi_bourges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{F7918DB6-62EF-48DD-BA2B-CE213045F091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3401AE44-50ED-4F56-B4B9-EE802157FB83}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="8_{F7918DB6-62EF-48DD-BA2B-CE213045F091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F26ED358-050B-4839-969D-6744BA71C24F}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -299,7 +299,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -396,6 +396,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -919,6 +927,9 @@
                 <c:pt idx="2" formatCode="0%">
                   <c:v>0.92</c:v>
                 </c:pt>
+                <c:pt idx="3" formatCode="0%">
+                  <c:v>1</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -988,6 +999,9 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0.38</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1322,6 +1336,9 @@
                 <c:pt idx="2">
                   <c:v>0.84199999999999997</c:v>
                 </c:pt>
+                <c:pt idx="3" formatCode="0.00%">
+                  <c:v>0.99199999999999999</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1391,6 +1408,9 @@
                 </c:pt>
                 <c:pt idx="2" formatCode="0.0%">
                   <c:v>0.82399999999999995</c:v>
+                </c:pt>
+                <c:pt idx="3" formatCode="0.00%">
+                  <c:v>0.93140000000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2799,7 +2819,9 @@
       <c r="D3" s="10">
         <v>0.92</v>
       </c>
-      <c r="E3" s="10"/>
+      <c r="E3" s="10">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="11" t="s">
@@ -2814,7 +2836,9 @@
       <c r="D4" s="12">
         <v>0.38</v>
       </c>
-      <c r="E4" s="12"/>
+      <c r="E4" s="12">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
@@ -2856,7 +2880,9 @@
       <c r="D8" s="23">
         <v>0.84199999999999997</v>
       </c>
-      <c r="E8" s="10"/>
+      <c r="E8" s="31">
+        <v>0.99199999999999999</v>
+      </c>
     </row>
     <row r="9" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
@@ -2871,7 +2897,9 @@
       <c r="D9" s="30">
         <v>0.82399999999999995</v>
       </c>
-      <c r="E9" s="12"/>
+      <c r="E9" s="32">
+        <v>0.93140000000000001</v>
+      </c>
     </row>
     <row r="10" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">

</xml_diff>